<commit_message>
feat(tools): add table-based change extraction to diff parser
Add normalize_change_type() and extract_changes_from_table() methods
to parse change information from HTML tables with change type keywords.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/document/output/diff_report.xlsx
+++ b/document/output/diff_report.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1856,6 +1856,259 @@
       </c>
       <c r="E60" s="2" t="inlineStr"/>
     </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>未知章节</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>描述:统一API入口</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>未知章节</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>删除</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>描述:被OAuth2.0替代</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>未知章节</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>修改</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>描述:升级到HikariCP</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>未知章节</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>删除</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>描述:性能监控工具包，已内置</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>未知章节</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>描述:新版监控代理</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>未知章节</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>修改</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>描述:安装脚本更新</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>未知章节</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>删除</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>描述:旧版工具集，不再维护</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>未知章节</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>描述:新版仪表盘</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>未知章节</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>删除</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>application.properties | /etc/app/application.properties</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>未知章节</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>application.yml | /etc/app/application.yml</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>未知章节</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>修改</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>logback.xml | /etc/app/logback.xml</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(tools): add chapter filtering options to diff parser
Add include_chapters and skip_chapters parameters to allow selective parsing:
- --chapters: only parse specified chapters (e.g., "5" or "5.1,5.2")
- --skip: skip specified chapters (e.g., "1,2")
- Support chapter number extraction and flexible matching

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/document/output/diff_report.xlsx
+++ b/document/output/diff_report.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1017,75 +1017,6 @@
       </c>
       <c r="E28" s="2" t="inlineStr"/>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>5.1.1 安装包变更</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>perf.tar.gz</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>性能监控工具包，已内置</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>5.1.1 安装包变更</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>legacy-tools.zip</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>旧版工具集，不再维护</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>5.1.2 配置文件变更</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>application.properties</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>/etc/app/application.properties</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1097,7 +1028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1640,75 +1571,6 @@
       </c>
       <c r="E27" s="2" t="inlineStr"/>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>5.1.1 安装包变更</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>agent-v2.0.jar</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>新版监控代理</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>5.1.1 安装包变更</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>dashboard-v2.war</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>新版仪表盘</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>5.1.2 配置文件变更</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>application.yml</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>/etc/app/application.yml</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1720,7 +1582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1936,52 +1798,6 @@
       </c>
       <c r="E10" s="2" t="inlineStr"/>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>5.1.1 安装包变更</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>setup.sh</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>安装脚本更新</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>5.1.2 配置文件变更</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>logback.xml</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>/etc/app/logback.xml</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(document): add separate impact column to diff report
Add dedicated "影响说明" (impact) field as a separate column in the diff report output. This improves clarity by separating impact descriptions from general change descriptions.

Changes:
- Extract impact field separately from change descriptions in diff_parser.py
- Update Excel output to include impact column with adjusted column widths
- Update HTML report table structure to display impact information
- Adjust field order in diff_validator.py to match new schema

This enhancement makes it easier to distinguish between the nature of a change and its impact on the system.

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/document/output/diff_report.xlsx
+++ b/document/output/diff_report.xlsx
@@ -455,14 +455,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,15 +479,20 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>影响说明</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>描述</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>验证状态</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -499,17 +505,18 @@
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>V1.0</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -518,17 +525,18 @@
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>旧版报表系统</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -537,17 +545,18 @@
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>邮件提醒功能</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -556,17 +565,18 @@
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>本地文件导入</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -575,17 +585,18 @@
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>config.properties</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -594,17 +605,18 @@
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>localhost</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -613,17 +625,18 @@
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -632,17 +645,18 @@
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -651,17 +665,18 @@
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>8080</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -670,17 +685,18 @@
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr"/>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>9090</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -689,17 +705,18 @@
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr"/>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>/opt/scripts/start.sh</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -708,17 +725,18 @@
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr"/>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>/opt/scripts/stop.sh</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -727,17 +745,18 @@
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr"/>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>JDK 8</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -746,17 +765,18 @@
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr"/>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>5.1.47</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -765,17 +785,18 @@
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr"/>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>5.0</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -784,17 +805,18 @@
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr"/>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -803,17 +825,18 @@
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr"/>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -822,17 +845,18 @@
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr"/>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>已移除</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -841,17 +865,18 @@
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr"/>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>旧服务</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -860,17 +885,18 @@
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr"/>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr"/>
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>旧版本配置</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -879,17 +905,18 @@
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr"/>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>旧服务</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -898,17 +925,18 @@
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr"/>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>旧版客户端兼容性问题</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -922,12 +950,13 @@
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -940,17 +969,18 @@
           <t>perf.tar.gz</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>性能监控工具包，已内置</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -963,17 +993,18 @@
           <t>legacy-tools.zip</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>旧版工具集，不再维护</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -987,12 +1018,13 @@
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr"/>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1010,12 +1042,93 @@
           <t>被OAuth2.0替代</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>5.1.1 安装包变更</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>perf.tar.gz</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>性能监控工具包，已内置</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>/opt/packages/perf.tar.gz</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>5.1.1 安装包变更</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>legacy-tools.zip</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>旧版工具集，不再维护</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>/opt/packages/legacy-tools.zip</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>5.1.2 配置文件变更</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>application.properties</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr"/>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>/etc/app/application.properties</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1028,14 +1141,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1051,15 +1165,20 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>影响说明</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>描述</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>验证状态</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -1072,17 +1191,18 @@
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>V2.0</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1091,17 +1211,18 @@
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>微服务架构</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1110,17 +1231,18 @@
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Excel、PDF、CSV</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1129,17 +1251,18 @@
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>config.yaml</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1148,17 +1271,18 @@
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>db-cluster.internal</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1167,17 +1291,18 @@
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>DEBUG</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1186,17 +1311,18 @@
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1205,17 +1331,18 @@
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>8081</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1224,17 +1351,18 @@
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>9091</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1243,17 +1371,18 @@
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr"/>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>/opt/scripts/start-service.sh</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1262,17 +1391,18 @@
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr"/>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>/opt/scripts/stop-service.sh</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1281,17 +1411,18 @@
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr"/>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>JDK 11</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1300,17 +1431,18 @@
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr"/>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>8.0.33</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1319,17 +1451,18 @@
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr"/>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>7.0</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1338,17 +1471,18 @@
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr"/>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1357,17 +1491,18 @@
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr"/>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>JDK 11</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1376,17 +1511,18 @@
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr"/>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>新版本安装脚本</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1395,17 +1531,18 @@
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr"/>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>config.yaml</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1414,17 +1551,18 @@
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr"/>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>新服务</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1433,17 +1571,18 @@
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr"/>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr"/>
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>新服务</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1452,17 +1591,18 @@
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr"/>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>需要5分钟初始化</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1476,12 +1616,13 @@
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr"/>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1494,17 +1635,18 @@
           <t>agent-v2.0.jar</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>新版监控代理</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1517,17 +1659,18 @@
           <t>dashboard-v2.war</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>新版仪表盘</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1541,12 +1684,13 @@
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1564,12 +1708,93 @@
           <t>统一API入口</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>5.1.1 安装包变更</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>agent-v2.0.jar</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>新版监控代理</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>/opt/packages/agent-v2.0.jar</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>5.1.1 安装包变更</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>dashboard-v2.war</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>新版仪表盘</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>/opt/packages/dashboard-v2.war</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>5.1.2 配置文件变更</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>application.yml</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>/etc/app/application.yml</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1582,14 +1807,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1605,15 +1831,20 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
+          <t>影响说明</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>描述</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>验证状态</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -1626,17 +1857,18 @@
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>系统升级过程中的所有变更</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1645,17 +1877,18 @@
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>UI优化，支持扫码登录</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1664,17 +1897,18 @@
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>增加模糊匹配和历史记录</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1683,17 +1917,18 @@
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>/opt/scripts/backup.sh</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1702,17 +1937,18 @@
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>配置项名称发生变化</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1726,12 +1962,13 @@
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1744,17 +1981,18 @@
           <t>setup.sh</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>安装脚本更新</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1768,12 +2006,13 @@
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1791,12 +2030,65 @@
           <t>升级到HikariCP</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>待验证</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>5.1.1 安装包变更</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>setup.sh</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>安装脚本更新</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>/opt/setup.sh</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>5.1.2 配置文件变更</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>logback.xml</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>/etc/app/logback.xml</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
refactor(document): reorganize HTML report layout
- Move total summary section above navigation tabs
- Remove sheet title headers from each sheet section
- Simplify sheet sections to only show filter buttons
- Update sheet-filters CSS with proper padding and center alignment
- Update diff_report.xlsx with validation results

This creates a cleaner layout with global summary at the top,
followed by navigation, then the filtered content for each sheet.

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/document/output/diff_report.xlsx
+++ b/document/output/diff_report.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +57,12 @@
         <bgColor rgb="00F57C00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8E6C9"/>
+        <bgColor rgb="00C8E6C9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -76,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -88,6 +94,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1066,14 +1075,14 @@
           <t>性能监控工具包，已内置</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>/opt/packages/perf.tar.gz</t>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>待验证</t>
+          <t>删除项（无法验证路径，符合预期）</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr"/>
@@ -1094,14 +1103,14 @@
           <t>旧版工具集，不再维护</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>/opt/packages/legacy-tools.zip</t>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>待验证</t>
+          <t>删除项（无法验证路径，符合预期）</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr"/>
@@ -1734,12 +1743,12 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>/opt/packages/agent-v2.0.jar</t>
+          <t>跳过</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>待验证</t>
+          <t>无法从描述中提取文件路径</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr"/>
@@ -1762,12 +1771,12 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>/opt/packages/dashboard-v2.war</t>
+          <t>跳过</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>待验证</t>
+          <t>无法从描述中提取文件路径</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2056,12 +2065,12 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>/opt/setup.sh</t>
+          <t>跳过</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>待验证</t>
+          <t>无法从描述中提取文件路径</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>

</xml_diff>